<commit_message>
chore: add .gitkeep to main folders and Alternative, fix merge BTP cross-search and no-photo fallback
</commit_message>
<xml_diff>
--- a/logs/merge_skipped.xlsx
+++ b/logs/merge_skipped.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Skipped Files" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skipped Files" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -61,7 +58,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,11 +424,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="101" customWidth="1" min="1" max="1"/>
-    <col width="131" customWidth="1" min="2" max="2"/>
+    <col width="106" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -455,459 +452,493 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN CATU DAYA 1 BULANAN_Cilebut.pdf</t>
+          <t>04-01-2025_PERAWATAN PERALATAN CTC CTS 1 BULANAN_Cilebut.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: CLT, CLT, CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:34</t>
+          <t>2026-07-14 17:46:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN PERALATAN CTC CTS 1 BULANAN_Cilebut.pdf</t>
+          <t>25-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Bogor.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: PANEL DISPLAY DALWAS PERKA CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:39</t>
+          <t>2026-07-14 17:46:09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Cilebut (2).pdf</t>
+          <t>17-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bojonggede-Cilebut.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:46</t>
+          <t>2026-07-14 17:46:15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Cilebut.pdf</t>
+          <t>23-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Batutulis.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: INTERLOCKING ELEKTRIK SIL-02 (HIMA) CLT, PANEL PELAYANAN VDU 1 CLT, PANEL PELAYANAN VDU 2 CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:46</t>
+          <t>2026-07-14 17:46:16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Maseng.pdf</t>
+          <t>24-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cilebut-Bogor (2).pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: ER TELKOM MSG</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:47</t>
+          <t>2026-07-14 17:46:16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>21-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Cigombong.pdf</t>
+          <t>24-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cilebut-Bogor.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: ER TELKOM CGB</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:50</t>
+          <t>2026-07-14 17:46:16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Batutulis.pdf</t>
+          <t>25-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogor (2).pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: ER TELKOM BTT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:50</t>
+          <t>2026-07-14 17:46:16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27-01-2025_PERAWATAN PERALATAN DALAM PERSINYALAN ELEKTRIK 1 BULANAN_Ciomas.pdf</t>
+          <t>25-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogor-Batutulis.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: TOWER COS</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:51</t>
+          <t>2026-07-14 17:46:17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI STASIUN 1 BULANAN_Cilebut.pdf</t>
+          <t>25-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogor.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:52</t>
+          <t>2026-07-14 17:46:17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI STASIUN 1 BULANAN_Ciomas.pdf</t>
+          <t>26-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogor-Batutulis.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: ER RADIO CIOMAS</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-13 22:47:56</t>
+          <t>2026-07-14 17:46:17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bojonggede-Cilebut.pdf</t>
+          <t>26-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogorpaledang-Batutulis.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: JPL 26N BJD-CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:03</t>
+          <t>2026-07-14 17:46:17</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>24-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cilebut-Bogor (2).pdf</t>
+          <t>26-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Bogorpaledang.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: 28 BOO-CLT, 28 BOO-CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:04</t>
+          <t>2026-07-14 17:46:18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cilebut-Bogor.pdf</t>
+          <t>30-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cigombong-Cicurug (2).pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: 27 BOO-CLT, 27 BOO-CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:04</t>
+          <t>2026-07-14 17:46:18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cilebut.pdf</t>
+          <t>30-01-2025_PERAWATAN PERALATAN TELEKOMUNIKASI DI PINTU PERLINTASAN 1 BULANAN_Cigombong-Cicurug.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:09</t>
+          <t>2026-07-14 17:46:18</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Batutulis-Maseng.pdf</t>
+          <t>07-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Bogor (3).pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO ER TELKOM MSG</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:09</t>
+          <t>2026-07-14 17:46:25</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>17-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cilebut.pdf</t>
+          <t>07-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 26N CLT-BJD</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:12</t>
+          <t>2026-07-14 17:46:25</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>21-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cigombong-Cicurug.pdf</t>
+          <t>08-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (2).pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO ER TELKOM CGB</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:12</t>
+          <t>2026-07-14 17:46:26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>21-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cigombong.pdf</t>
+          <t>08-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (3).pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: IB CGB</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:13</t>
+          <t>2026-07-14 17:46:26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Batutulis (2).pdf</t>
+          <t>08-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 11 BTT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:13</t>
+          <t>2026-07-14 17:46:26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Bogor.pdf</t>
+          <t>10-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (2).pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO ER TELKOM BTT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:14</t>
+          <t>2026-07-14 17:46:27</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>24-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Bogor (2).pdf</t>
+          <t>10-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (3).pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 28 BOO-CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:15</t>
+          <t>2026-07-14 17:46:27</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>24-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Bogor.pdf</t>
+          <t>10-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (4).pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 27 BOO-CLT</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:15</t>
+          <t>2026-07-14 17:46:27</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>25-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Bogor (2).pdf</t>
+          <t>10-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor.pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 01 BOO, FO JPL 02 BOO</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:15</t>
+          <t>2026-07-14 17:46:28</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>26-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Bogor.pdf</t>
+          <t>12-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (2).pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 04 BOO-BOP, FO JPL BNR BOO-BOP, FO JPL 07 BOO-BOP</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:16</t>
+          <t>2026-07-14 17:46:28</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>27-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Ciomas.pdf</t>
+          <t>12-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor (3).pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: IB COS</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:17</t>
+          <t>2026-07-14 17:46:28</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>30-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cigombong (2).pdf</t>
+          <t>12-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Cilebut-Bogor.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 16 CGB</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:17</t>
+          <t>2026-07-14 17:46:28</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>30-01-2025_PERAWATAN SERAT OPTIK 1 BULANAN_Cigombong.pdf</t>
+          <t>14-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Bojonggede-Cilebut (2).pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>skipped: missing photos for assets: FO JPL 15 CGB</t>
+          <t>skipped: no photos found for any identifier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-07-13 22:48:17</t>
+          <t>2026-07-14 17:46:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Bojonggede-Cilebut.pdf</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>skipped: no photos found for any identifier</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:46:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>30-01-2025_PERAWATAN PERAGA SINYAL ELEKTRIK 1 BULANAN_Batutulis-Maseng.pdf</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>skipped: no photos found for any identifier</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-07-14 17:46:36</t>
         </is>
       </c>
     </row>

</xml_diff>